<commit_message>
Set up all the data retrieval stuff
</commit_message>
<xml_diff>
--- a/src/resources/RecentIPOLockupExpirations.xlsx
+++ b/src/resources/RecentIPOLockupExpirations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffsando/Desktop/options-tracker/src/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D13635FA-37AF-264E-9722-7DF30D22933D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E67CBD-DBC1-DC4C-BB36-F8ACFEBB0AE8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30700" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{B6968569-0E6B-1748-89BA-8E171A76172E}"/>
   </bookViews>
@@ -19,11 +19,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -841,10 +836,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
         <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>2</v>
       </c>
       <c r="C13" s="1">
         <v>18.350000000000001</v>

</xml_diff>